<commit_message>
[Fix - Monster Data] Jellymong 공격력 조정 ( 10 -> 5 )
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Monster.xlsx
+++ b/JsonConverter/ExcelFiles/Monster.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.12458"/>
+  <x:fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.12581"/>
   <x:workbookPr date1904="0" showBorderUnselectedTables="1" filterPrivacy="0" promptedSolutions="0" showInkAnnotation="1" backupFile="0" saveExternalLinkValues="1" codeName="ThisWorkbook" hidePivotFieldList="0" allowRefreshQuery="0" publishItems="0" checkCompatibility="0" autoCompressPictures="1" refreshAllConnections="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" Requires="x15">
@@ -21,10 +21,55 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PrefabPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>일반 공격 스킬 배율</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>스킬 공격의 배율 리스트(나중에 스킬 데이터로 빠질 수 있다)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NormalAtkDamage</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몬스터 설명 (도감용)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몬스터 표기용 Icon</x:t>
+  </x:si>
+  <x:si>
+    <x:t>mob_jellymong_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>젤리몽</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>float[]</x:t>
+  </x:si>
+  <x:si>
     <x:t>float</x:t>
   </x:si>
   <x:si>
-    <x:t>float[]</x:t>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
   </x:si>
   <x:si>
     <x:t>BaseHp</x:t>
@@ -33,70 +78,25 @@
     <x:t>기본 공격력</x:t>
   </x:si>
   <x:si>
+    <x:t>BaseAtk</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몬스터를 우선 프리팹으로 구현</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Jellymong</x:t>
+  </x:si>
+  <x:si>
+    <x:t>말랑한 몸을 이용해 적에게 바디박치기를 하는 몬스터</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Monster_Jelltmong</x:t>
+  </x:si>
+  <x:si>
     <x:t>SkillAtkMultipleList</x:t>
-  </x:si>
-  <x:si>
-    <x:t>말랑한 몸을 이용해 적에게 바디박치기를 하는 몬스터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>스킬 공격의 배율 리스트(나중에 스킬 데이터로 빠질 수 있다)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseAtk</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>젤리몽</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몬스터를 우선 프리팹으로 구현</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Jellymong</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PrefabPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>mob_jellymong_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몬스터 표기용 Icon</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몬스터 설명 (도감용)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Monster_Jelltmong</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NormalAtkDamage</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>일반 공격 스킬 배율</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -916,56 +916,56 @@
   <x:sheetData>
     <x:row r="1" spans="1:9" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D1" s="1"/>
       <x:c r="E1" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F1" s="1" t="s">
-        <x:v>25</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G1" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H1" s="2" t="s">
-        <x:v>20</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="I1" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:10" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>0</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>1</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="I2" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J2" s="1"/>
     </x:row>
@@ -974,46 +974,46 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B3" s="12" t="s">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C3" s="12" t="s">
-        <x:v>18</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D3" s="12" t="s">
-        <x:v>2</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E3" s="12" t="s">
-        <x:v>7</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F3" s="12" t="s">
-        <x:v>23</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G3" s="12" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H3" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H3" s="14" t="s">
-        <x:v>17</x:v>
-      </x:c>
       <x:c r="I3" s="14" t="s">
-        <x:v>15</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J3" s="15"/>
     </x:row>
     <x:row r="4" spans="1:19" ht="15.75" customHeight="1">
       <x:c r="A4" s="4" t="s">
-        <x:v>19</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="4" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s">
-        <x:v>5</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D4" s="4">
         <x:v>50</x:v>
       </x:c>
       <x:c r="E4" s="4">
-        <x:v>10</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F4" s="4">
         <x:v>1</x:v>
@@ -1022,10 +1022,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H4" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I4" s="5" t="s">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="J4" s="16"/>
       <x:c r="K4" s="5"/>

</xml_diff>

<commit_message>
[Monster Data] 데이터 추가 - 튀김맨
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Monster.xlsx
+++ b/JsonConverter/ExcelFiles/Monster.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="18852" windowHeight="6720"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="18852" windowHeight="6792"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId4"/>
@@ -19,7 +19,73 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+  <x:si>
+    <x:t>Icon/Icon_Fryman</x:t>
+  </x:si>
+  <x:si>
+    <x:t>스킬 공격의 배율 리스트(나중에 스킬 데이터로 빠질 수 있다)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>젤리몽</x:t>
+  </x:si>
+  <x:si>
+    <x:t>튀김맨</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몬스터를 우선 프리팹으로 구현</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Jellymong</x:t>
+  </x:si>
+  <x:si>
+    <x:t>float[]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>float</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 공격력</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BaseHp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BaseAtk</x:t>
+  </x:si>
+  <x:si>
+    <x:t>mob_fryman_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>mob_jellymong_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NormalAtkDamage</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몬스터 표기용 Icon</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몬스터 설명 (도감용)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
   <x:si>
     <x:t>캐릭터 고유 ID</x:t>
   </x:si>
@@ -30,73 +96,22 @@
     <x:t>일반 공격 스킬 배율</x:t>
   </x:si>
   <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
     <x:t>IconPath</x:t>
   </x:si>
   <x:si>
-    <x:t>스킬 공격의 배율 리스트(나중에 스킬 데이터로 빠질 수 있다)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NormalAtkDamage</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몬스터 설명 (도감용)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몬스터 표기용 Icon</x:t>
-  </x:si>
-  <x:si>
-    <x:t>mob_jellymong_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>젤리몽</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>float[]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>float</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseHp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 공격력</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseAtk</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몬스터를 우선 프리팹으로 구현</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Jellymong</x:t>
-  </x:si>
-  <x:si>
-    <x:t>말랑한 몸을 이용해 적에게 바디박치기를 하는 몬스터</x:t>
+    <x:t>말랑한 몸을 이용해 바디박치기를 하는 몬스터</x:t>
   </x:si>
   <x:si>
     <x:t>2DObject/Monster_Jelltmong</x:t>
   </x:si>
   <x:si>
     <x:t>SkillAtkMultipleList</x:t>
+  </x:si>
+  <x:si>
+    <x:t>날카로운 창을 이용해 공격하는 몬스터</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2DObject/Monster_Fryman</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -916,98 +931,98 @@
   <x:sheetData>
     <x:row r="1" spans="1:9" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>0</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
-        <x:v>7</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D1" s="1"/>
       <x:c r="E1" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F1" s="1" t="s">
-        <x:v>2</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="G1" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H1" s="2" t="s">
-        <x:v>8</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="I1" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:10" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H2" s="1" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E2" s="1" t="s">
+      <x:c r="I2" s="1" t="s">
         <x:v>12</x:v>
-      </x:c>
-      <x:c r="F2" s="1" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="G2" s="1" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="H2" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="I2" s="1" t="s">
-        <x:v>15</x:v>
       </x:c>
       <x:c r="J2" s="1"/>
     </x:row>
     <x:row r="3" spans="1:10" s="13" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="12" t="s">
-        <x:v>11</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="12" t="s">
-        <x:v>20</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C3" s="12" t="s">
-        <x:v>3</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D3" s="12" t="s">
-        <x:v>17</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E3" s="12" t="s">
-        <x:v>19</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F3" s="12" t="s">
-        <x:v>6</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G3" s="12" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H3" s="14" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="H3" s="14" t="s">
-        <x:v>4</x:v>
-      </x:c>
       <x:c r="I3" s="14" t="s">
-        <x:v>1</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="J3" s="15"/>
     </x:row>
     <x:row r="4" spans="1:19" ht="15.75" customHeight="1">
       <x:c r="A4" s="4" t="s">
-        <x:v>9</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B4" s="4" t="s">
-        <x:v>10</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D4" s="4">
         <x:v>50</x:v>
@@ -1022,10 +1037,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H4" s="5" t="s">
-        <x:v>22</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="I4" s="5" t="s">
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="J4" s="16"/>
       <x:c r="K4" s="5"/>
@@ -1039,15 +1054,33 @@
       <x:c r="S4" s="5"/>
     </x:row>
     <x:row r="5" spans="1:19" ht="15.75" customHeight="1">
-      <x:c r="A5" s="4"/>
-      <x:c r="B5" s="6"/>
-      <x:c r="C5" s="6"/>
-      <x:c r="D5" s="6"/>
-      <x:c r="E5" s="6"/>
-      <x:c r="F5" s="6"/>
-      <x:c r="G5" s="6"/>
-      <x:c r="H5" s="5"/>
-      <x:c r="I5" s="5"/>
+      <x:c r="A5" s="4" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D5" s="6">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E5" s="6">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F5" s="6">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="6">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H5" s="5" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="5" t="s">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="J5" s="5"/>
       <x:c r="K5" s="5"/>
       <x:c r="L5" s="5"/>

</xml_diff>

<commit_message>
[Add - Monster Data] RewardExp 데이터 필드 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Monster.xlsx
+++ b/JsonConverter/ExcelFiles/Monster.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="18852" windowHeight="6792"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="18828" windowHeight="6792"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId4"/>
@@ -19,99 +19,105 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+  <x:si>
+    <x:t>RewardExp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>보상 경험치</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>젤리몽</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>튀김맨</x:t>
+  </x:si>
+  <x:si>
+    <x:t>스킬 공격의 배율 리스트(나중에 스킬 데이터로 빠질 수 있다)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BaseHp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>float[]</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BaseAtk</x:t>
+  </x:si>
+  <x:si>
+    <x:t>float</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 공격력</x:t>
+  </x:si>
   <x:si>
     <x:t>Icon/Icon_Fryman</x:t>
   </x:si>
   <x:si>
-    <x:t>스킬 공격의 배율 리스트(나중에 스킬 데이터로 빠질 수 있다)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>젤리몽</x:t>
-  </x:si>
-  <x:si>
-    <x:t>튀김맨</x:t>
-  </x:si>
-  <x:si>
     <x:t>몬스터를 우선 프리팹으로 구현</x:t>
   </x:si>
   <x:si>
     <x:t>Icon/Icon_Jellymong</x:t>
   </x:si>
   <x:si>
-    <x:t>float[]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>float</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 공격력</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseHp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseAtk</x:t>
+    <x:t>mob_jellymong_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몬스터 설명 (도감용)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>몬스터 표기용 Icon</x:t>
   </x:si>
   <x:si>
     <x:t>mob_fryman_1</x:t>
   </x:si>
   <x:si>
-    <x:t>mob_jellymong_1</x:t>
-  </x:si>
-  <x:si>
     <x:t>NormalAtkDamage</x:t>
   </x:si>
   <x:si>
-    <x:t>몬스터 표기용 Icon</x:t>
-  </x:si>
-  <x:si>
-    <x:t>몬스터 설명 (도감용)</x:t>
+    <x:t>캐릭터 고유 ID</x:t>
   </x:si>
   <x:si>
     <x:t>Description</x:t>
   </x:si>
   <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
+    <x:t>일반 공격 스킬 배율</x:t>
   </x:si>
   <x:si>
     <x:t>PrefabPath</x:t>
   </x:si>
   <x:si>
-    <x:t>일반 공격 스킬 배율</x:t>
-  </x:si>
-  <x:si>
     <x:t>IconPath</x:t>
   </x:si>
   <x:si>
+    <x:t>2DObject/Monster_Fryman</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SkillAtkMultipleList</x:t>
+  </x:si>
+  <x:si>
+    <x:t>날카로운 창을 이용해 공격하는 몬스터</x:t>
+  </x:si>
+  <x:si>
     <x:t>말랑한 몸을 이용해 바디박치기를 하는 몬스터</x:t>
   </x:si>
   <x:si>
     <x:t>2DObject/Monster_Jelltmong</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SkillAtkMultipleList</x:t>
-  </x:si>
-  <x:si>
-    <x:t>날카로운 창을 이용해 공격하는 몬스터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2DObject/Monster_Fryman</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -914,115 +920,124 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:S35"/>
+  <x:dimension ref="A1:T35"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="19.453125" style="3" customWidth="1"/>
     <x:col min="2" max="2" width="19.54296875" style="3" customWidth="1"/>
     <x:col min="3" max="3" width="63.22265625" style="3" customWidth="1"/>
-    <x:col min="4" max="5" width="23.22265625" style="3" customWidth="1"/>
-    <x:col min="6" max="6" width="25.109375" style="3" customWidth="1"/>
-    <x:col min="7" max="7" width="52.22265625" style="3" customWidth="1"/>
-    <x:col min="8" max="8" width="23.22265625" style="3" customWidth="1"/>
-    <x:col min="9" max="9" width="30.54296875" style="3" customWidth="1"/>
-    <x:col min="10" max="10" width="26.54296875" style="3" customWidth="1"/>
-    <x:col min="11" max="16384" width="12.54296875" style="3"/>
+    <x:col min="4" max="6" width="23.22265625" style="3" customWidth="1"/>
+    <x:col min="7" max="7" width="25.109375" style="3" customWidth="1"/>
+    <x:col min="8" max="8" width="52.22265625" style="3" customWidth="1"/>
+    <x:col min="9" max="9" width="23.22265625" style="3" customWidth="1"/>
+    <x:col min="10" max="10" width="30.54296875" style="3" customWidth="1"/>
+    <x:col min="11" max="11" width="26.54296875" style="3" customWidth="1"/>
+    <x:col min="12" max="16384" width="12.54296875" style="3"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:9" ht="15.75" customHeight="1">
+    <x:row r="1" spans="1:10" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D1" s="1"/>
       <x:c r="E1" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I1" s="2" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J1" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:11" ht="13.199999999999999">
+      <x:c r="A2" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H2" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="J2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K2" s="1"/>
+    </x:row>
+    <x:row r="3" spans="1:11" s="13" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A3" s="12" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F1" s="1" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="G1" s="1" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H1" s="2" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I1" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:10" ht="13.199999999999999">
-      <x:c r="A2" s="1" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
+      <x:c r="F3" s="12" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H3" s="12" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="I3" s="14" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="J3" s="14" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="K3" s="15"/>
+    </x:row>
+    <x:row r="4" spans="1:20" ht="15.75" customHeight="1">
+      <x:c r="A4" s="4" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F2" s="1" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="G2" s="1" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H2" s="1" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="I2" s="1" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="J2" s="1"/>
-    </x:row>
-    <x:row r="3" spans="1:10" s="13" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A3" s="12" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="D3" s="12" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E3" s="12" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F3" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="G3" s="12" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="H3" s="14" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="I3" s="14" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="J3" s="15"/>
-    </x:row>
-    <x:row r="4" spans="1:19" ht="15.75" customHeight="1">
-      <x:c r="A4" s="4" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B4" s="4" t="s">
-        <x:v>4</x:v>
-      </x:c>
       <x:c r="C4" s="4" t="s">
-        <x:v>26</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D4" s="4">
         <x:v>50</x:v>
@@ -1031,19 +1046,21 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="F4" s="4">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G4" s="4">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G4" s="4">
+      <x:c r="H4" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H4" s="5" t="s">
-        <x:v>7</x:v>
-      </x:c>
       <x:c r="I4" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="J4" s="16"/>
-      <x:c r="K4" s="5"/>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="J4" s="5" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="K4" s="16"/>
       <x:c r="L4" s="5"/>
       <x:c r="M4" s="5"/>
       <x:c r="N4" s="5"/>
@@ -1052,16 +1069,17 @@
       <x:c r="Q4" s="5"/>
       <x:c r="R4" s="5"/>
       <x:c r="S4" s="5"/>
-    </x:row>
-    <x:row r="5" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T4" s="5"/>
+    </x:row>
+    <x:row r="5" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A5" s="4" t="s">
-        <x:v>16</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D5" s="6">
         <x:v>60</x:v>
@@ -1070,18 +1088,20 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="F5" s="6">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G5" s="6">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G5" s="6">
+      <x:c r="H5" s="6">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H5" s="5" t="s">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="I5" s="5" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="J5" s="5"/>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="J5" s="5" t="s">
+        <x:v>28</x:v>
+      </x:c>
       <x:c r="K5" s="5"/>
       <x:c r="L5" s="5"/>
       <x:c r="M5" s="5"/>
@@ -1091,8 +1111,9 @@
       <x:c r="Q5" s="5"/>
       <x:c r="R5" s="5"/>
       <x:c r="S5" s="5"/>
-    </x:row>
-    <x:row r="6" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T5" s="5"/>
+    </x:row>
+    <x:row r="6" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A6" s="6"/>
       <x:c r="B6" s="6"/>
       <x:c r="C6" s="6"/>
@@ -1100,7 +1121,7 @@
       <x:c r="E6" s="6"/>
       <x:c r="F6" s="6"/>
       <x:c r="G6" s="6"/>
-      <x:c r="H6" s="5"/>
+      <x:c r="H6" s="6"/>
       <x:c r="I6" s="5"/>
       <x:c r="J6" s="5"/>
       <x:c r="K6" s="5"/>
@@ -1112,8 +1133,9 @@
       <x:c r="Q6" s="5"/>
       <x:c r="R6" s="5"/>
       <x:c r="S6" s="5"/>
-    </x:row>
-    <x:row r="7" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T6" s="5"/>
+    </x:row>
+    <x:row r="7" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A7" s="4"/>
       <x:c r="B7" s="4"/>
       <x:c r="C7" s="4"/>
@@ -1121,7 +1143,7 @@
       <x:c r="E7" s="4"/>
       <x:c r="F7" s="4"/>
       <x:c r="G7" s="4"/>
-      <x:c r="H7" s="5"/>
+      <x:c r="H7" s="4"/>
       <x:c r="I7" s="5"/>
       <x:c r="J7" s="5"/>
       <x:c r="K7" s="5"/>
@@ -1133,8 +1155,9 @@
       <x:c r="Q7" s="5"/>
       <x:c r="R7" s="5"/>
       <x:c r="S7" s="5"/>
-    </x:row>
-    <x:row r="8" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T7" s="5"/>
+    </x:row>
+    <x:row r="8" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A8" s="7"/>
       <x:c r="B8" s="7"/>
       <x:c r="C8" s="7"/>
@@ -1142,7 +1165,7 @@
       <x:c r="E8" s="7"/>
       <x:c r="F8" s="7"/>
       <x:c r="G8" s="7"/>
-      <x:c r="H8" s="5"/>
+      <x:c r="H8" s="7"/>
       <x:c r="I8" s="5"/>
       <x:c r="J8" s="5"/>
       <x:c r="K8" s="5"/>
@@ -1154,8 +1177,9 @@
       <x:c r="Q8" s="5"/>
       <x:c r="R8" s="5"/>
       <x:c r="S8" s="5"/>
-    </x:row>
-    <x:row r="9" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T8" s="5"/>
+    </x:row>
+    <x:row r="9" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A9" s="7"/>
       <x:c r="B9" s="7"/>
       <x:c r="C9" s="7"/>
@@ -1163,7 +1187,7 @@
       <x:c r="E9" s="7"/>
       <x:c r="F9" s="7"/>
       <x:c r="G9" s="7"/>
-      <x:c r="H9" s="5"/>
+      <x:c r="H9" s="7"/>
       <x:c r="I9" s="5"/>
       <x:c r="J9" s="5"/>
       <x:c r="K9" s="5"/>
@@ -1175,8 +1199,9 @@
       <x:c r="Q9" s="5"/>
       <x:c r="R9" s="5"/>
       <x:c r="S9" s="5"/>
-    </x:row>
-    <x:row r="10" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T9" s="5"/>
+    </x:row>
+    <x:row r="10" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A10" s="1"/>
       <x:c r="B10" s="1"/>
       <x:c r="C10" s="1"/>
@@ -1184,7 +1209,7 @@
       <x:c r="E10" s="1"/>
       <x:c r="F10" s="1"/>
       <x:c r="G10" s="1"/>
-      <x:c r="H10" s="5"/>
+      <x:c r="H10" s="1"/>
       <x:c r="I10" s="5"/>
       <x:c r="J10" s="5"/>
       <x:c r="K10" s="5"/>
@@ -1196,8 +1221,9 @@
       <x:c r="Q10" s="5"/>
       <x:c r="R10" s="5"/>
       <x:c r="S10" s="5"/>
-    </x:row>
-    <x:row r="11" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T10" s="5"/>
+    </x:row>
+    <x:row r="11" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A11" s="1"/>
       <x:c r="B11" s="1"/>
       <x:c r="C11" s="1"/>
@@ -1205,7 +1231,7 @@
       <x:c r="E11" s="1"/>
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
-      <x:c r="H11" s="5"/>
+      <x:c r="H11" s="1"/>
       <x:c r="I11" s="5"/>
       <x:c r="J11" s="5"/>
       <x:c r="K11" s="5"/>
@@ -1217,8 +1243,9 @@
       <x:c r="Q11" s="5"/>
       <x:c r="R11" s="5"/>
       <x:c r="S11" s="5"/>
-    </x:row>
-    <x:row r="12" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T11" s="5"/>
+    </x:row>
+    <x:row r="12" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A12" s="7"/>
       <x:c r="B12" s="7"/>
       <x:c r="C12" s="7"/>
@@ -1226,7 +1253,7 @@
       <x:c r="E12" s="7"/>
       <x:c r="F12" s="7"/>
       <x:c r="G12" s="7"/>
-      <x:c r="H12" s="5"/>
+      <x:c r="H12" s="7"/>
       <x:c r="I12" s="5"/>
       <x:c r="J12" s="5"/>
       <x:c r="K12" s="5"/>
@@ -1238,8 +1265,9 @@
       <x:c r="Q12" s="5"/>
       <x:c r="R12" s="5"/>
       <x:c r="S12" s="5"/>
-    </x:row>
-    <x:row r="13" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T12" s="5"/>
+    </x:row>
+    <x:row r="13" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A13" s="4"/>
       <x:c r="B13" s="4"/>
       <x:c r="C13" s="4"/>
@@ -1247,7 +1275,7 @@
       <x:c r="E13" s="4"/>
       <x:c r="F13" s="4"/>
       <x:c r="G13" s="4"/>
-      <x:c r="H13" s="5"/>
+      <x:c r="H13" s="4"/>
       <x:c r="I13" s="5"/>
       <x:c r="J13" s="5"/>
       <x:c r="K13" s="5"/>
@@ -1259,8 +1287,9 @@
       <x:c r="Q13" s="5"/>
       <x:c r="R13" s="5"/>
       <x:c r="S13" s="5"/>
-    </x:row>
-    <x:row r="14" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T13" s="5"/>
+    </x:row>
+    <x:row r="14" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A14" s="1"/>
       <x:c r="B14" s="1"/>
       <x:c r="C14" s="1"/>
@@ -1268,7 +1297,7 @@
       <x:c r="E14" s="1"/>
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
-      <x:c r="H14" s="5"/>
+      <x:c r="H14" s="1"/>
       <x:c r="I14" s="5"/>
       <x:c r="J14" s="5"/>
       <x:c r="K14" s="5"/>
@@ -1280,8 +1309,9 @@
       <x:c r="Q14" s="5"/>
       <x:c r="R14" s="5"/>
       <x:c r="S14" s="5"/>
-    </x:row>
-    <x:row r="15" spans="1:19" ht="15.75" customHeight="1">
+      <x:c r="T14" s="5"/>
+    </x:row>
+    <x:row r="15" spans="1:20" ht="15.75" customHeight="1">
       <x:c r="A15" s="1"/>
       <x:c r="B15" s="1"/>
       <x:c r="C15" s="1"/>
@@ -1289,7 +1319,7 @@
       <x:c r="E15" s="1"/>
       <x:c r="F15" s="1"/>
       <x:c r="G15" s="1"/>
-      <x:c r="H15" s="5"/>
+      <x:c r="H15" s="1"/>
       <x:c r="I15" s="5"/>
       <x:c r="J15" s="5"/>
       <x:c r="K15" s="5"/>
@@ -1301,8 +1331,9 @@
       <x:c r="Q15" s="5"/>
       <x:c r="R15" s="5"/>
       <x:c r="S15" s="5"/>
-    </x:row>
-    <x:row r="16" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="T15" s="5"/>
+    </x:row>
+    <x:row r="16" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A16" s="8"/>
       <x:c r="B16" s="8"/>
       <x:c r="C16" s="8"/>
@@ -1310,8 +1341,9 @@
       <x:c r="E16" s="8"/>
       <x:c r="F16" s="8"/>
       <x:c r="G16" s="8"/>
-    </x:row>
-    <x:row r="17" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H16" s="8"/>
+    </x:row>
+    <x:row r="17" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A17" s="9"/>
       <x:c r="B17" s="9"/>
       <x:c r="C17" s="9"/>
@@ -1319,8 +1351,9 @@
       <x:c r="E17" s="8"/>
       <x:c r="F17" s="8"/>
       <x:c r="G17" s="8"/>
-    </x:row>
-    <x:row r="18" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H17" s="8"/>
+    </x:row>
+    <x:row r="18" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A18" s="9"/>
       <x:c r="B18" s="9"/>
       <x:c r="C18" s="9"/>
@@ -1328,8 +1361,9 @@
       <x:c r="E18" s="8"/>
       <x:c r="F18" s="8"/>
       <x:c r="G18" s="8"/>
-    </x:row>
-    <x:row r="19" spans="1:9" ht="15.75" customHeight="1">
+      <x:c r="H18" s="8"/>
+    </x:row>
+    <x:row r="19" spans="1:10" ht="15.75" customHeight="1">
       <x:c r="A19" s="9"/>
       <x:c r="B19" s="9"/>
       <x:c r="C19" s="9"/>
@@ -1337,10 +1371,11 @@
       <x:c r="E19" s="8"/>
       <x:c r="F19" s="8"/>
       <x:c r="G19" s="8"/>
-      <x:c r="H19" s="5"/>
+      <x:c r="H19" s="8"/>
       <x:c r="I19" s="5"/>
-    </x:row>
-    <x:row r="20" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="J19" s="5"/>
+    </x:row>
+    <x:row r="20" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A20" s="9"/>
       <x:c r="B20" s="9"/>
       <x:c r="C20" s="9"/>
@@ -1348,8 +1383,9 @@
       <x:c r="E20" s="8"/>
       <x:c r="F20" s="8"/>
       <x:c r="G20" s="8"/>
-    </x:row>
-    <x:row r="21" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H20" s="8"/>
+    </x:row>
+    <x:row r="21" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A21" s="9"/>
       <x:c r="B21" s="9"/>
       <x:c r="C21" s="9"/>
@@ -1357,8 +1393,9 @@
       <x:c r="E21" s="8"/>
       <x:c r="F21" s="8"/>
       <x:c r="G21" s="8"/>
-    </x:row>
-    <x:row r="22" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H21" s="8"/>
+    </x:row>
+    <x:row r="22" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A22" s="9"/>
       <x:c r="B22" s="9"/>
       <x:c r="C22" s="9"/>
@@ -1366,8 +1403,9 @@
       <x:c r="E22" s="8"/>
       <x:c r="F22" s="8"/>
       <x:c r="G22" s="8"/>
-    </x:row>
-    <x:row r="23" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H22" s="8"/>
+    </x:row>
+    <x:row r="23" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A23" s="9"/>
       <x:c r="B23" s="9"/>
       <x:c r="C23" s="9"/>
@@ -1375,8 +1413,9 @@
       <x:c r="E23" s="8"/>
       <x:c r="F23" s="8"/>
       <x:c r="G23" s="8"/>
-    </x:row>
-    <x:row r="24" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H23" s="8"/>
+    </x:row>
+    <x:row r="24" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A24" s="9"/>
       <x:c r="B24" s="9"/>
       <x:c r="C24" s="9"/>
@@ -1384,8 +1423,9 @@
       <x:c r="E24" s="8"/>
       <x:c r="F24" s="8"/>
       <x:c r="G24" s="8"/>
-    </x:row>
-    <x:row r="25" spans="1:9" ht="15.75" customHeight="1">
+      <x:c r="H24" s="8"/>
+    </x:row>
+    <x:row r="25" spans="1:10" ht="15.75" customHeight="1">
       <x:c r="A25" s="9"/>
       <x:c r="B25" s="9"/>
       <x:c r="C25" s="9"/>
@@ -1393,9 +1433,10 @@
       <x:c r="E25" s="8"/>
       <x:c r="F25" s="8"/>
       <x:c r="G25" s="8"/>
-      <x:c r="I25" s="5"/>
-    </x:row>
-    <x:row r="26" spans="1:9" ht="15.75" customHeight="1">
+      <x:c r="H25" s="8"/>
+      <x:c r="J25" s="5"/>
+    </x:row>
+    <x:row r="26" spans="1:10" ht="15.75" customHeight="1">
       <x:c r="A26" s="10"/>
       <x:c r="B26" s="10"/>
       <x:c r="C26" s="10"/>
@@ -1403,9 +1444,10 @@
       <x:c r="E26" s="10"/>
       <x:c r="F26" s="10"/>
       <x:c r="G26" s="10"/>
-      <x:c r="I26" s="5"/>
-    </x:row>
-    <x:row r="27" spans="1:9" ht="15.75" customHeight="1">
+      <x:c r="H26" s="10"/>
+      <x:c r="J26" s="5"/>
+    </x:row>
+    <x:row r="27" spans="1:10" ht="15.75" customHeight="1">
       <x:c r="A27" s="10"/>
       <x:c r="B27" s="10"/>
       <x:c r="C27" s="10"/>
@@ -1413,9 +1455,10 @@
       <x:c r="E27" s="10"/>
       <x:c r="F27" s="10"/>
       <x:c r="G27" s="10"/>
-      <x:c r="I27" s="5"/>
-    </x:row>
-    <x:row r="28" spans="1:9" ht="15.75" customHeight="1">
+      <x:c r="H27" s="10"/>
+      <x:c r="J27" s="5"/>
+    </x:row>
+    <x:row r="28" spans="1:10" ht="15.75" customHeight="1">
       <x:c r="A28" s="10"/>
       <x:c r="B28" s="10"/>
       <x:c r="C28" s="10"/>
@@ -1423,9 +1466,10 @@
       <x:c r="E28" s="10"/>
       <x:c r="F28" s="10"/>
       <x:c r="G28" s="10"/>
-      <x:c r="I28" s="5"/>
-    </x:row>
-    <x:row r="29" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H28" s="10"/>
+      <x:c r="J28" s="5"/>
+    </x:row>
+    <x:row r="29" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A29" s="10"/>
       <x:c r="B29" s="10"/>
       <x:c r="C29" s="10"/>
@@ -1433,8 +1477,9 @@
       <x:c r="E29" s="10"/>
       <x:c r="F29" s="10"/>
       <x:c r="G29" s="10"/>
-    </x:row>
-    <x:row r="30" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H29" s="10"/>
+    </x:row>
+    <x:row r="30" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A30" s="10"/>
       <x:c r="B30" s="10"/>
       <x:c r="C30" s="10"/>
@@ -1442,8 +1487,9 @@
       <x:c r="E30" s="10"/>
       <x:c r="F30" s="10"/>
       <x:c r="G30" s="10"/>
-    </x:row>
-    <x:row r="31" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H30" s="10"/>
+    </x:row>
+    <x:row r="31" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A31" s="10"/>
       <x:c r="B31" s="10"/>
       <x:c r="C31" s="10"/>
@@ -1451,8 +1497,9 @@
       <x:c r="E31" s="10"/>
       <x:c r="F31" s="10"/>
       <x:c r="G31" s="10"/>
-    </x:row>
-    <x:row r="32" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H31" s="10"/>
+    </x:row>
+    <x:row r="32" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A32" s="11"/>
       <x:c r="B32" s="11"/>
       <x:c r="C32" s="11"/>
@@ -1460,8 +1507,9 @@
       <x:c r="E32" s="11"/>
       <x:c r="F32" s="11"/>
       <x:c r="G32" s="11"/>
-    </x:row>
-    <x:row r="33" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H32" s="11"/>
+    </x:row>
+    <x:row r="33" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A33" s="11"/>
       <x:c r="B33" s="11"/>
       <x:c r="C33" s="11"/>
@@ -1469,8 +1517,9 @@
       <x:c r="E33" s="11"/>
       <x:c r="F33" s="11"/>
       <x:c r="G33" s="11"/>
-    </x:row>
-    <x:row r="34" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H33" s="11"/>
+    </x:row>
+    <x:row r="34" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A34" s="11"/>
       <x:c r="B34" s="11"/>
       <x:c r="C34" s="11"/>
@@ -1478,8 +1527,9 @@
       <x:c r="E34" s="11"/>
       <x:c r="F34" s="11"/>
       <x:c r="G34" s="11"/>
-    </x:row>
-    <x:row r="35" spans="1:7" ht="15.75" customHeight="1">
+      <x:c r="H34" s="11"/>
+    </x:row>
+    <x:row r="35" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A35" s="11"/>
       <x:c r="B35" s="11"/>
       <x:c r="C35" s="11"/>
@@ -1487,6 +1537,7 @@
       <x:c r="E35" s="11"/>
       <x:c r="F35" s="11"/>
       <x:c r="G35" s="11"/>
+      <x:c r="H35" s="11"/>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1"/>
     <x:row r="37" ht="15.75" customHeight="1"/>

</xml_diff>